<commit_message>
Prepare English v0.1-beta web application
</commit_message>
<xml_diff>
--- a/BarkodListe/verified-export.xlsx
+++ b/BarkodListe/verified-export.xlsx
@@ -7,7 +7,7 @@
     <sheet name="HepsiJet" sheetId="2" r:id="rId2"/>
     <sheet name="Tex" sheetId="3" r:id="rId3"/>
     <sheet name="Aras" sheetId="4" r:id="rId4"/>
-    <sheet name="Bilinmeyen" sheetId="5" r:id="rId5"/>
+    <sheet name="Unknown" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -409,10 +409,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Barkod</v>
+        <v>Barcode</v>
       </c>
       <c r="B1" t="str">
-        <v>Tekrar sayısı</v>
+        <v>Quantity</v>
       </c>
     </row>
     <row r="2">
@@ -448,10 +448,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Barkod</v>
+        <v>Barcode</v>
       </c>
       <c r="B1" t="str">
-        <v>Tekrar sayısı</v>
+        <v>Quantity</v>
       </c>
     </row>
     <row r="2">
@@ -495,10 +495,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Barkod</v>
+        <v>Barcode</v>
       </c>
       <c r="B1" t="str">
-        <v>Tekrar sayısı</v>
+        <v>Quantity</v>
       </c>
     </row>
     <row r="2">
@@ -526,10 +526,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Barkod</v>
+        <v>Barcode</v>
       </c>
       <c r="B1" t="str">
-        <v>Tekrar sayısı</v>
+        <v>Quantity</v>
       </c>
     </row>
     <row r="2">
@@ -581,10 +581,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Barkod</v>
+        <v>Barcode</v>
       </c>
       <c r="B1" t="str">
-        <v>Tekrar sayısı</v>
+        <v>Quantity</v>
       </c>
     </row>
     <row r="2">

</xml_diff>